<commit_message>
refactor: remove quality score, update target matching logic, and refine pipeline summary details
</commit_message>
<xml_diff>
--- a/webapp/static/example_targets.xlsx
+++ b/webapp/static/example_targets.xlsx
@@ -49,94 +49,94 @@
     <t>CHEMBL1910</t>
   </si>
   <si>
-    <t>Maltase-glucoamylase</t>
-  </si>
-  <si>
-    <t>ATP-binding cassette sub-family C member 9</t>
-  </si>
-  <si>
-    <t>cGMP-specific 3',5'-cyclic phosphodiesterase</t>
-  </si>
-  <si>
-    <t>Voltage-dependent T-type calcium channel subunit alpha-1H</t>
-  </si>
-  <si>
-    <t>Dihydrofolate reductase</t>
-  </si>
-  <si>
-    <t>Tyrosine-protein kinase ABL1</t>
-  </si>
-  <si>
-    <t>Epidermal growth factor receptor</t>
-  </si>
-  <si>
-    <t>Prothrombin</t>
-  </si>
-  <si>
-    <t>Plasminogen</t>
-  </si>
-  <si>
-    <t>Adenosine deaminase</t>
-  </si>
-  <si>
-    <t>O43451</t>
-  </si>
-  <si>
-    <t>O60706</t>
-  </si>
-  <si>
-    <t>O76074</t>
-  </si>
-  <si>
-    <t>O95180</t>
-  </si>
-  <si>
-    <t>P00374</t>
-  </si>
-  <si>
-    <t>P00519</t>
-  </si>
-  <si>
-    <t>P00533</t>
-  </si>
-  <si>
-    <t>P00734</t>
-  </si>
-  <si>
-    <t>P00747</t>
-  </si>
-  <si>
-    <t>P00813</t>
-  </si>
-  <si>
-    <t>MGAM</t>
-  </si>
-  <si>
-    <t>ABCC9</t>
-  </si>
-  <si>
-    <t>PDE5A</t>
-  </si>
-  <si>
-    <t>CACNA1H</t>
-  </si>
-  <si>
-    <t>DHFR</t>
-  </si>
-  <si>
-    <t>ABL1</t>
-  </si>
-  <si>
-    <t>EGFR</t>
-  </si>
-  <si>
-    <t>F2</t>
-  </si>
-  <si>
-    <t>PLG</t>
-  </si>
-  <si>
-    <t>ADA</t>
+    <t>Carbonic anhydrase 2</t>
+  </si>
+  <si>
+    <t>Antithrombin-III</t>
+  </si>
+  <si>
+    <t>Troponin C, slow skeletal and cardiac muscles</t>
+  </si>
+  <si>
+    <t>Estrogen receptor</t>
+  </si>
+  <si>
+    <t>Plasma kallikrein</t>
+  </si>
+  <si>
+    <t>3-hydroxy-3-methylglutaryl-coenzyme A reductase</t>
+  </si>
+  <si>
+    <t>Glucocorticoid receptor</t>
+  </si>
+  <si>
+    <t>Thymidylate synthase</t>
+  </si>
+  <si>
+    <t>Sodium/potassium-transporting ATPase subunit alpha-1</t>
+  </si>
+  <si>
+    <t>Aldehyde dehydrogenase, mitochondrial</t>
+  </si>
+  <si>
+    <t>P05106</t>
+  </si>
+  <si>
+    <t>P05108</t>
+  </si>
+  <si>
+    <t>P68371</t>
+  </si>
+  <si>
+    <t>P05556</t>
+  </si>
+  <si>
+    <t>P06213</t>
+  </si>
+  <si>
+    <t>P06401</t>
+  </si>
+  <si>
+    <t>P07099</t>
+  </si>
+  <si>
+    <t>P07101</t>
+  </si>
+  <si>
+    <t>P07202</t>
+  </si>
+  <si>
+    <t>P07327</t>
+  </si>
+  <si>
+    <t>PRSS1</t>
+  </si>
+  <si>
+    <t>ADRB2</t>
+  </si>
+  <si>
+    <t>CHRM2</t>
+  </si>
+  <si>
+    <t>NR3C2</t>
+  </si>
+  <si>
+    <t>ITGA2B</t>
+  </si>
+  <si>
+    <t>ADRB1</t>
+  </si>
+  <si>
+    <t>HTR1A</t>
+  </si>
+  <si>
+    <t>ADRA2A</t>
+  </si>
+  <si>
+    <t>POLA1</t>
+  </si>
+  <si>
+    <t>ALOX5</t>
   </si>
 </sst>
 </file>

</xml_diff>